<commit_message>
final tables and figures manipulation
</commit_message>
<xml_diff>
--- a/Results/betareg_sensitivity_Peninsula_excel.xlsx
+++ b/Results/betareg_sensitivity_Peninsula_excel.xlsx
@@ -1,21 +1,74 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\OneDrive\Desktop\Artigos_coauthor\Iberian_plants\Extinction_dynamics_Iberic\Results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A20A82-4FDF-4BF6-8E79-EF5030AF680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+  <si>
+    <t>term</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>mean_estimate</t>
+  </si>
+  <si>
+    <t>sd_estimate</t>
+  </si>
+  <si>
+    <t>mean_p</t>
+  </si>
+  <si>
+    <t>prop_significant</t>
+  </si>
+  <si>
+    <t>Intercept</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Intermediate</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Corrected age</t>
+  </si>
+  <si>
+    <t>Diversification rates</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Peninsula</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,10 +105,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -63,13 +119,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +171,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +205,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +240,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,291 +416,222 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>scenario</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mean_estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>sd_estimate</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>median_estimate</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mean_p</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>prop_significant</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>-1.82643020783224</v>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>0.06753470117899842</v>
+        <v>-1.8264302078322401</v>
       </c>
       <c r="E2">
-        <v>-1.816799832759616</v>
+        <v>6.7534701178998416E-2</v>
       </c>
       <c r="F2">
-        <v>1.264596693039004E-136</v>
+        <v>1.2645966930390041E-136</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-      <c r="C3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>6.3057978630394152E-3</v>
+      </c>
+      <c r="E3">
+        <v>1.117920469254665E-3</v>
+      </c>
+      <c r="F3">
+        <v>3.1582361622425073E-2</v>
+      </c>
+      <c r="G3">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>-0.1020174374362901</v>
+      </c>
+      <c r="E4">
+        <v>5.9196836507810047E-2</v>
+      </c>
+      <c r="F4">
+        <v>0.58977475609576013</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5">
         <v>-1.843863812589976</v>
       </c>
-      <c r="D3">
-        <v>0.06666895166980545</v>
-      </c>
-      <c r="E3">
-        <v>-1.833448935853421</v>
-      </c>
-      <c r="F3">
-        <v>1.614779837516115E-92</v>
-      </c>
-      <c r="G3">
+      <c r="E5">
+        <v>6.6668951669805451E-2</v>
+      </c>
+      <c r="F5">
+        <v>1.6147798375161149E-92</v>
+      </c>
+      <c r="G5">
         <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>-1.871499428195137</v>
-      </c>
-      <c r="D4">
-        <v>0.0684335435985628</v>
-      </c>
-      <c r="E4">
-        <v>-1.864834078713368</v>
-      </c>
-      <c r="F4">
-        <v>2.892828750614522E-60</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Corrected age</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>0.006305797863039415</v>
-      </c>
-      <c r="D5">
-        <v>0.001117920469254665</v>
-      </c>
-      <c r="E5">
-        <v>0.00622237832099018</v>
-      </c>
-      <c r="F5">
-        <v>0.03158236162242507</v>
-      </c>
-      <c r="G5">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Corrected age</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>0.01076531436458521</v>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" t="s">
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>0.00188370094272728</v>
+        <v>1.0765314364585211E-2</v>
       </c>
       <c r="E6">
-        <v>0.01089272048187503</v>
+        <v>1.88370094272728E-3</v>
       </c>
       <c r="F6">
-        <v>0.08003787758281428</v>
+        <v>8.0037877582814276E-2</v>
       </c>
       <c r="G6">
         <v>0.32</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Corrected age</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>0.02007268213502426</v>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" t="s">
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>0.003906363202867098</v>
+        <v>-8.2850216945780236E-2</v>
       </c>
       <c r="E7">
-        <v>0.01989170535660111</v>
+        <v>5.9449770348962587E-2</v>
       </c>
       <c r="F7">
+        <v>0.66755299630853759</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>-1.8714994281951369</v>
+      </c>
+      <c r="E8">
+        <v>6.8433543598562796E-2</v>
+      </c>
+      <c r="F8">
+        <v>2.8928287506145221E-60</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>2.0072682135024261E-2</v>
+      </c>
+      <c r="E9">
+        <v>3.9063632028670976E-3</v>
+      </c>
+      <c r="F9">
         <v>0.1237624564699816</v>
       </c>
-      <c r="G7">
+      <c r="G9">
         <v>0.09</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Diversification rates</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>-0.1020174374362901</v>
-      </c>
-      <c r="D8">
-        <v>0.05919683650781005</v>
-      </c>
-      <c r="E8">
-        <v>-0.1000480550628166</v>
-      </c>
-      <c r="F8">
-        <v>0.5897747560957601</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Diversification rates</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Intermediate</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>-0.08285021694578024</v>
-      </c>
-      <c r="D9">
-        <v>0.05944977034896259</v>
-      </c>
-      <c r="E9">
-        <v>-0.08208710776722847</v>
-      </c>
-      <c r="F9">
-        <v>0.6675529963085376</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Diversification rates</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>-0.05806665602821981</v>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" t="s">
+        <v>11</v>
       </c>
       <c r="D10">
-        <v>0.06320186608267088</v>
+        <v>-5.806665602821981E-2</v>
       </c>
       <c r="E10">
-        <v>-0.05496973027031631</v>
+        <v>6.3201866082670879E-2</v>
       </c>
       <c r="F10">
-        <v>0.7444111976825145</v>
+        <v>0.74441119768251451</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>